<commit_message>
a few bug fixes
</commit_message>
<xml_diff>
--- a/readme_files/bootloader_summary.xlsx
+++ b/readme_files/bootloader_summary.xlsx
@@ -345,9 +345,6 @@
     <t>SDIO_F446ZE_fatfs-stm32-master</t>
   </si>
   <si>
-    <t>3E78</t>
-  </si>
-  <si>
     <t>BTT Octopus V1.1</t>
   </si>
   <si>
@@ -355,6 +352,9 @@
   </si>
   <si>
     <t>STM32F446ZE</t>
+  </si>
+  <si>
+    <t>3EC8</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1512,10 +1512,10 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C9" t="s">
         <v>29</v>
@@ -1774,16 +1774,16 @@
         <v>105</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D24" s="14">
         <v>8004000</v>
       </c>
       <c r="E24" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="H24" s="12" t="s">
         <v>107</v>
-      </c>
-      <c r="H24" s="12" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.45">

</xml_diff>